<commit_message>
feat(eval): v2.13.2 age-banded 1RM standards - Elie's confirmed numbers replace placeholders
Elie (2026-07-14, in-session): 18-39 keeps the approved 5-level thresholds;
40-49/50-59/60-69/70+ scale them by the decline factors from his age-range
tables (band benchmark / 18-39 benchmark, per lift per gender), rounded to
2 decimals - he confirmed this exact method ('the math u did is correct').
CHARTS_VERSION 2 -> 3; existing frozen evaluations keep their v2 scores,
only new evaluations use the banded tables.
Sanity: age-band boundary checks added (39/40 edge, 70+ rescore), frozen
chartsVersion assertion now tracks the constant. As-implemented xlsx
regenerated with confirmed status.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KYfRbDeceCWcZwMV9ikW4R
</commit_message>
<xml_diff>
--- a/docs/superpowers/artifacts/2026-07-06-1rm-battery/PT-1RM-Standards-As-Implemented.xlsx
+++ b/docs/superpowers/artifacts/2026-07-06-1rm-battery/PT-1RM-Standards-As-Implemented.xlsx
@@ -14,9 +14,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="47">
-  <si>
-    <t>1RM standards as implemented in the app (charts version 2) — generated 2026-07-13</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="129">
+  <si>
+    <t>1RM standards as implemented in the app (charts version 3) — generated 2026-07-14</t>
   </si>
   <si>
     <t/>
@@ -28,28 +28,13 @@
     <t>Example: 80 kg client benching 100 kg → ratio 1.25. "≥ N" = minimum ratio to earn that level.</t>
   </si>
   <si>
-    <t>IMPORTANT — THESE ARE PLACEHOLDERS. They are simplified from published adult strength</t>
-  </si>
-  <si>
-    <t>standards (ExRx.net / Kraemer &amp; Fleck-style tables). Please send YOUR numbers and we swap them in</t>
-  </si>
-  <si>
-    <t>(same as we did for sit &amp; reach in the old battery).</t>
-  </si>
-  <si>
-    <t>QUESTION 1 — AGE: right now ONE flat band applies to all ages. Should older clients get</t>
-  </si>
-  <si>
-    <t>easier thresholds? If yes, send age-banded values (e.g. 18-35 / 36-50 / 51+).</t>
-  </si>
-  <si>
-    <t>QUESTION 2 — the classification from the three lift scores is unchanged from your rule:</t>
-  </si>
-  <si>
-    <t>average of bench+squat+deadlift scores → 1-1.9 Beginner A · 2-2.9 Beginner B · 3-3.9 Intermediate A</t>
-  </si>
-  <si>
-    <t>· exactly 4 Intermediate B · above 4 Pro. Confirm this still applies to the 1RM battery.</t>
+    <t>STATUS: CONFIRMED BY ELIE 2026-07-14 (in-session). The 18-39 rows are the levels he</t>
+  </si>
+  <si>
+    <t>approved; the older age bands are those levels scaled down by the decline factors from</t>
+  </si>
+  <si>
+    <t>his age-range tables (each band’s benchmark ÷ the 18-39 benchmark, per lift, per gender).</t>
   </si>
   <si>
     <t>Reply with corrections and we update the app — old saved evaluations keep their frozen scores,</t>
@@ -82,7 +67,7 @@
     <t>Excellent (5)</t>
   </si>
   <si>
-    <t>ALL AGES</t>
+    <t>0-39</t>
   </si>
   <si>
     <t>&lt; 0.75</t>
@@ -100,6 +85,75 @@
     <t>≥ 1.65</t>
   </si>
   <si>
+    <t>40-49</t>
+  </si>
+  <si>
+    <t>&lt; 0.69</t>
+  </si>
+  <si>
+    <t>≥ 0.69</t>
+  </si>
+  <si>
+    <t>≥ 0.92</t>
+  </si>
+  <si>
+    <t>≥ 1.24</t>
+  </si>
+  <si>
+    <t>≥ 1.51</t>
+  </si>
+  <si>
+    <t>50-59</t>
+  </si>
+  <si>
+    <t>&lt; 0.63</t>
+  </si>
+  <si>
+    <t>≥ 0.63</t>
+  </si>
+  <si>
+    <t>≥ 0.83</t>
+  </si>
+  <si>
+    <t>≥ 1.13</t>
+  </si>
+  <si>
+    <t>≥ 1.38</t>
+  </si>
+  <si>
+    <t>60-69</t>
+  </si>
+  <si>
+    <t>&lt; 0.53</t>
+  </si>
+  <si>
+    <t>≥ 0.53</t>
+  </si>
+  <si>
+    <t>≥ 0.71</t>
+  </si>
+  <si>
+    <t>≥ 0.96</t>
+  </si>
+  <si>
+    <t>≥ 1.17</t>
+  </si>
+  <si>
+    <t>70+</t>
+  </si>
+  <si>
+    <t>&lt; 0.44</t>
+  </si>
+  <si>
+    <t>≥ 0.44</t>
+  </si>
+  <si>
+    <t>≥ 0.58</t>
+  </si>
+  <si>
+    <t>≥ 0.79</t>
+  </si>
+  <si>
     <t>FEMALE</t>
   </si>
   <si>
@@ -118,6 +172,54 @@
     <t>≥ 1.1</t>
   </si>
   <si>
+    <t>&lt; 0.45</t>
+  </si>
+  <si>
+    <t>≥ 0.45</t>
+  </si>
+  <si>
+    <t>≥ 0.82</t>
+  </si>
+  <si>
+    <t>&lt; 0.4</t>
+  </si>
+  <si>
+    <t>≥ 0.4</t>
+  </si>
+  <si>
+    <t>≥ 0.56</t>
+  </si>
+  <si>
+    <t>≥ 0.72</t>
+  </si>
+  <si>
+    <t>≥ 0.88</t>
+  </si>
+  <si>
+    <t>&lt; 0.35</t>
+  </si>
+  <si>
+    <t>≥ 0.35</t>
+  </si>
+  <si>
+    <t>≥ 0.49</t>
+  </si>
+  <si>
+    <t>≥ 0.62</t>
+  </si>
+  <si>
+    <t>≥ 0.76</t>
+  </si>
+  <si>
+    <t>&lt; 0.28</t>
+  </si>
+  <si>
+    <t>≥ 0.28</t>
+  </si>
+  <si>
+    <t>≥ 0.39</t>
+  </si>
+  <si>
     <t>Squat — 1RM ÷ bodyweight ratio, one flat age band (see Read Me).</t>
   </si>
   <si>
@@ -136,9 +238,90 @@
     <t>≥ 2.5</t>
   </si>
   <si>
+    <t>&lt; 1.13</t>
+  </si>
+  <si>
+    <t>≥ 1.8</t>
+  </si>
+  <si>
+    <t>≥ 2.25</t>
+  </si>
+  <si>
+    <t>&lt; 1</t>
+  </si>
+  <si>
+    <t>≥ 1.2</t>
+  </si>
+  <si>
+    <t>≥ 1.6</t>
+  </si>
+  <si>
+    <t>&lt; 0.88</t>
+  </si>
+  <si>
+    <t>≥ 1.05</t>
+  </si>
+  <si>
+    <t>≥ 1.4</t>
+  </si>
+  <si>
+    <t>≥ 1.75</t>
+  </si>
+  <si>
+    <t>&lt; 0.71</t>
+  </si>
+  <si>
+    <t>≥ 0.85</t>
+  </si>
+  <si>
+    <t>≥ 1.42</t>
+  </si>
+  <si>
     <t>≥ 1.85</t>
   </si>
   <si>
+    <t>&lt; 0.68</t>
+  </si>
+  <si>
+    <t>≥ 0.68</t>
+  </si>
+  <si>
+    <t>≥ 1.67</t>
+  </si>
+  <si>
+    <t>&lt; 0.6</t>
+  </si>
+  <si>
+    <t>≥ 0.6</t>
+  </si>
+  <si>
+    <t>≥ 0.8</t>
+  </si>
+  <si>
+    <t>≥ 1.48</t>
+  </si>
+  <si>
+    <t>&lt; 0.52</t>
+  </si>
+  <si>
+    <t>≥ 0.52</t>
+  </si>
+  <si>
+    <t>≥ 1.3</t>
+  </si>
+  <si>
+    <t>&lt; 0.41</t>
+  </si>
+  <si>
+    <t>≥ 0.41</t>
+  </si>
+  <si>
+    <t>≥ 0.55</t>
+  </si>
+  <si>
+    <t>≥ 1.02</t>
+  </si>
+  <si>
     <t>Deadlift — 1RM ÷ bodyweight ratio, one flat age band (see Read Me).</t>
   </si>
   <si>
@@ -148,13 +331,76 @@
     <t>≥ 3</t>
   </si>
   <si>
-    <t>&lt; 1</t>
-  </si>
-  <si>
-    <t>≥ 1.75</t>
-  </si>
-  <si>
-    <t>≥ 2.25</t>
+    <t>&lt; 1.37</t>
+  </si>
+  <si>
+    <t>≥ 1.37</t>
+  </si>
+  <si>
+    <t>≥ 1.83</t>
+  </si>
+  <si>
+    <t>≥ 2.29</t>
+  </si>
+  <si>
+    <t>≥ 2.74</t>
+  </si>
+  <si>
+    <t>&lt; 1.24</t>
+  </si>
+  <si>
+    <t>≥ 1.66</t>
+  </si>
+  <si>
+    <t>≥ 2.07</t>
+  </si>
+  <si>
+    <t>≥ 2.49</t>
+  </si>
+  <si>
+    <t>&lt; 1.07</t>
+  </si>
+  <si>
+    <t>≥ 1.07</t>
+  </si>
+  <si>
+    <t>≥ 1.43</t>
+  </si>
+  <si>
+    <t>≥ 1.79</t>
+  </si>
+  <si>
+    <t>≥ 2.14</t>
+  </si>
+  <si>
+    <t>&lt; 0.9</t>
+  </si>
+  <si>
+    <t>&lt; 0.92</t>
+  </si>
+  <si>
+    <t>≥ 1.15</t>
+  </si>
+  <si>
+    <t>≥ 1.61</t>
+  </si>
+  <si>
+    <t>&lt; 0.8</t>
+  </si>
+  <si>
+    <t>&lt; 0.7</t>
+  </si>
+  <si>
+    <t>≥ 1.23</t>
+  </si>
+  <si>
+    <t>≥ 1.58</t>
+  </si>
+  <si>
+    <t>&lt; 0.58</t>
+  </si>
+  <si>
+    <t>≥ 1.01</t>
   </si>
 </sst>
 </file>
@@ -539,7 +785,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -600,41 +846,6 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>13</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -643,7 +854,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="6" width="18" customWidth="1"/>
@@ -651,97 +862,257 @@
   <sheetData>
     <row r="1" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" t="s">
         <v>16</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" t="s">
         <v>22</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>23</v>
       </c>
-      <c r="C5" t="s">
+      <c r="B6" t="s">
         <v>24</v>
       </c>
-      <c r="D5" t="s">
+      <c r="C6" t="s">
         <v>25</v>
       </c>
-      <c r="E5" t="s">
+      <c r="D6" t="s">
         <v>26</v>
       </c>
-      <c r="F5" t="s">
+      <c r="E6" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="F6" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="E8" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="F8" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="B9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" t="s">
+        <v>43</v>
+      </c>
+      <c r="D9" t="s">
+        <v>44</v>
+      </c>
+      <c r="E9" t="s">
+        <v>45</v>
+      </c>
+      <c r="F9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" t="s">
+        <v>48</v>
+      </c>
+      <c r="D13" t="s">
+        <v>49</v>
+      </c>
+      <c r="E13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" t="s">
+        <v>53</v>
+      </c>
+      <c r="D14" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" t="s">
+        <v>54</v>
+      </c>
+      <c r="F14" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>29</v>
       </c>
-      <c r="C9" t="s">
-        <v>30</v>
-      </c>
-      <c r="D9" t="s">
-        <v>31</v>
-      </c>
-      <c r="E9" t="s">
-        <v>32</v>
-      </c>
-      <c r="F9" t="s">
-        <v>33</v>
+      <c r="B15" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" t="s">
+        <v>56</v>
+      </c>
+      <c r="D15" t="s">
+        <v>57</v>
+      </c>
+      <c r="E15" t="s">
+        <v>58</v>
+      </c>
+      <c r="F15" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" t="s">
+        <v>60</v>
+      </c>
+      <c r="C16" t="s">
+        <v>61</v>
+      </c>
+      <c r="D16" t="s">
+        <v>62</v>
+      </c>
+      <c r="E16" t="s">
+        <v>63</v>
+      </c>
+      <c r="F16" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17" t="s">
+        <v>65</v>
+      </c>
+      <c r="C17" t="s">
+        <v>66</v>
+      </c>
+      <c r="D17" t="s">
+        <v>67</v>
+      </c>
+      <c r="E17" t="s">
+        <v>48</v>
+      </c>
+      <c r="F17" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -752,7 +1123,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="6" width="18" customWidth="1"/>
@@ -760,97 +1131,257 @@
   <sheetData>
     <row r="1" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>34</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" t="s">
         <v>16</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>69</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>70</v>
       </c>
       <c r="D5" t="s">
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="E5" t="s">
-        <v>38</v>
+        <v>72</v>
       </c>
       <c r="F5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>28</v>
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" t="s">
+        <v>75</v>
+      </c>
+      <c r="F6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" t="s">
+        <v>77</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" t="s">
+        <v>78</v>
+      </c>
+      <c r="E7" t="s">
+        <v>79</v>
+      </c>
+      <c r="F7" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>80</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
+        <v>59</v>
       </c>
       <c r="D8" t="s">
-        <v>19</v>
+        <v>81</v>
       </c>
       <c r="E8" t="s">
-        <v>20</v>
+        <v>82</v>
       </c>
       <c r="F8" t="s">
-        <v>21</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="B9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" t="s">
+        <v>85</v>
+      </c>
+      <c r="E9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" t="s">
+        <v>20</v>
+      </c>
+      <c r="E13" t="s">
+        <v>71</v>
+      </c>
+      <c r="F13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>23</v>
       </c>
-      <c r="C9" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" t="s">
-        <v>25</v>
-      </c>
-      <c r="E9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F9" t="s">
-        <v>40</v>
+      <c r="B14" t="s">
+        <v>88</v>
+      </c>
+      <c r="C14" t="s">
+        <v>89</v>
+      </c>
+      <c r="D14" t="s">
+        <v>50</v>
+      </c>
+      <c r="E14" t="s">
+        <v>21</v>
+      </c>
+      <c r="F14" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" t="s">
+        <v>91</v>
+      </c>
+      <c r="C15" t="s">
+        <v>92</v>
+      </c>
+      <c r="D15" t="s">
+        <v>93</v>
+      </c>
+      <c r="E15" t="s">
+        <v>78</v>
+      </c>
+      <c r="F15" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" t="s">
+        <v>95</v>
+      </c>
+      <c r="C16" t="s">
+        <v>96</v>
+      </c>
+      <c r="D16" t="s">
+        <v>49</v>
+      </c>
+      <c r="E16" t="s">
+        <v>81</v>
+      </c>
+      <c r="F16" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17" t="s">
+        <v>98</v>
+      </c>
+      <c r="C17" t="s">
+        <v>99</v>
+      </c>
+      <c r="D17" t="s">
+        <v>100</v>
+      </c>
+      <c r="E17" t="s">
+        <v>32</v>
+      </c>
+      <c r="F17" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -861,7 +1392,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="6" width="18" customWidth="1"/>
@@ -869,97 +1400,257 @@
   <sheetData>
     <row r="1" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>41</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" t="s">
         <v>16</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>42</v>
+        <v>103</v>
       </c>
       <c r="C5" t="s">
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="D5" t="s">
-        <v>38</v>
+        <v>72</v>
       </c>
       <c r="E5" t="s">
-        <v>39</v>
+        <v>73</v>
       </c>
       <c r="F5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>28</v>
+        <v>104</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D6" t="s">
+        <v>107</v>
+      </c>
+      <c r="E6" t="s">
+        <v>108</v>
+      </c>
+      <c r="F6" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" t="s">
+        <v>111</v>
+      </c>
+      <c r="E7" t="s">
+        <v>112</v>
+      </c>
+      <c r="F7" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>114</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
+        <v>115</v>
       </c>
       <c r="D8" t="s">
-        <v>19</v>
+        <v>116</v>
       </c>
       <c r="E8" t="s">
-        <v>20</v>
+        <v>117</v>
       </c>
       <c r="F8" t="s">
-        <v>21</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="B9" t="s">
+        <v>119</v>
+      </c>
+      <c r="C9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" t="s">
+        <v>78</v>
+      </c>
+      <c r="E9" t="s">
+        <v>71</v>
+      </c>
+      <c r="F9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" t="s">
+        <v>77</v>
+      </c>
+      <c r="C13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" t="s">
+        <v>70</v>
+      </c>
+      <c r="E13" t="s">
+        <v>83</v>
+      </c>
+      <c r="F13" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" t="s">
+        <v>120</v>
+      </c>
+      <c r="C14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" t="s">
+        <v>121</v>
+      </c>
+      <c r="E14" t="s">
+        <v>122</v>
+      </c>
+      <c r="F14" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" t="s">
+        <v>123</v>
+      </c>
+      <c r="C15" t="s">
+        <v>93</v>
+      </c>
+      <c r="D15" t="s">
+        <v>20</v>
+      </c>
+      <c r="E15" t="s">
+        <v>82</v>
+      </c>
+      <c r="F15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" t="s">
+        <v>124</v>
+      </c>
+      <c r="C16" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16" t="s">
+        <v>59</v>
+      </c>
+      <c r="E16" t="s">
+        <v>125</v>
+      </c>
+      <c r="F16" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17" t="s">
+        <v>127</v>
+      </c>
+      <c r="C17" t="s">
         <v>44</v>
       </c>
-      <c r="C9" t="s">
-        <v>25</v>
-      </c>
-      <c r="D9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E9" t="s">
-        <v>45</v>
-      </c>
-      <c r="F9" t="s">
-        <v>46</v>
+      <c r="D17" t="s">
+        <v>58</v>
+      </c>
+      <c r="E17" t="s">
+        <v>128</v>
+      </c>
+      <c r="F17" t="s">
+        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>